<commit_message>
a little bit of additional work!
</commit_message>
<xml_diff>
--- a/descriptives_by_sensor_table.xlsx
+++ b/descriptives_by_sensor_table.xlsx
@@ -1472,7 +1472,7 @@
         <v>44</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="15" ht="NA" customHeight="1">
@@ -1675,7 +1675,7 @@
         <v>44</v>
       </c>
       <c r="I21" s="9" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22" ht="NA" customHeight="1">

</xml_diff>